<commit_message>
updated for compatibility with PLS-Dataset
</commit_message>
<xml_diff>
--- a/datasets/raw/SMILES_to_BigSMILES_Conversion_wo_block_copolymer_with_HSPs.xlsx
+++ b/datasets/raw/SMILES_to_BigSMILES_Conversion_wo_block_copolymer_with_HSPs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdehgha2\Desktop\phd-code\PLS-Dataset\datasets\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AC3AF2-1AC5-4665-8A4E-AC6F7687E4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C307596A-8FD0-4195-8615-45FCB9CE7E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structures" sheetId="1" r:id="rId1"/>
@@ -1167,9 +1167,6 @@
     <t>PFT3</t>
   </si>
   <si>
-    <t>*c4ccc3c2ccc(c1ccc(*)s1)cc2C(CCC[N+](C)(C)CC)(CCC[N+](C)(CC)CC)c3c4.[Br-].[Br-]</t>
-  </si>
-  <si>
     <t>{&lt;c1ccc2c(c1)C(CCC[N+](C)(C)CC)(CCC[N+](C)(CC)CC)c1cc(ccc12.[Br-].[Br-])c3ccc(s3)&gt;}</t>
   </si>
   <si>
@@ -1864,6 +1861,9 @@
   </si>
   <si>
     <t>[*]C1=CC2=C(C3=C(C(c4sc(CCCCCC)c(CCCCCC)c4)=C2S1)C=C(c5c(CCCCCCCC)cc(c(n6)sc7c6sc(c8sc([*])c(CCCCCCCC)c8)n7)s5)S3)c9sc(CCCCCC)c(CCCCCC)c9</t>
+  </si>
+  <si>
+    <t>*c1ccc2c(c1)C(CCC[N+](C)(C)CC)(CCC[N+](C)(C)CC)c1cc(-c3ccc(*)s3)ccc1-2.[Br-].[Br-]</t>
   </si>
 </sst>
 </file>
@@ -3265,24 +3265,24 @@
         <v>#VALUE!</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B23" t="e" vm="21">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="E23">
         <v>18.5</v>
@@ -3296,16 +3296,16 @@
     </row>
     <row r="24" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" t="e" vm="22">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B24" t="e" vm="22">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="E24">
         <v>18.3</v>
@@ -3319,16 +3319,16 @@
     </row>
     <row r="25" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="e" vm="23">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B25" t="e" vm="23">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="E25">
         <v>17.5</v>
@@ -3342,16 +3342,16 @@
     </row>
     <row r="26" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="e" vm="24">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B26" t="e" vm="24">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="E26">
         <v>18.3</v>
@@ -3365,30 +3365,30 @@
     </row>
     <row r="27" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" t="e" vm="25">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B27" t="e" vm="25">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="e" vm="26">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B28" t="e" vm="26">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="E28">
         <v>20.7</v>
@@ -3402,16 +3402,16 @@
     </row>
     <row r="29" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" t="e" vm="27">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B29" t="e" vm="27">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="E29">
         <v>18.600000000000001</v>
@@ -3425,16 +3425,16 @@
     </row>
     <row r="30" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" t="e" vm="28">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B30" t="e" vm="28">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="E30">
         <v>18.8</v>
@@ -3448,16 +3448,16 @@
     </row>
     <row r="31" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" t="e" vm="29">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B31" t="e" vm="29">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="E31">
         <v>19.100000000000001</v>
@@ -3471,16 +3471,16 @@
     </row>
     <row r="32" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" t="s">
         <v>95</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="E32">
         <v>18.7</v>
@@ -3494,16 +3494,16 @@
     </row>
     <row r="33" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" t="e" vm="30">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B33" t="e" vm="30">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="E33">
         <v>20.100000000000001</v>
@@ -3517,16 +3517,16 @@
     </row>
     <row r="34" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B34" t="e" vm="31">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B34" t="e" vm="31">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="E34">
         <v>17.100000000000001</v>
@@ -3540,16 +3540,16 @@
     </row>
     <row r="35" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" t="e" vm="32">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B35" t="e" vm="32">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="D35" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="E35">
         <v>19.100000000000001</v>
@@ -3563,16 +3563,16 @@
     </row>
     <row r="36" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" t="e" vm="33">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B36" t="e" vm="33">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="E36">
         <v>17.7</v>
@@ -3586,16 +3586,16 @@
     </row>
     <row r="37" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B37" t="e" vm="34">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B37" t="e" vm="34">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="E37">
         <v>17.399999999999999</v>
@@ -3609,31 +3609,31 @@
     </row>
     <row r="38" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="B38" t="e" vm="35">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="J38" s="6"/>
     </row>
     <row r="39" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B39" t="e" vm="36">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B39" t="e" vm="36">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="E39">
         <v>18.899999999999999</v>
@@ -3647,16 +3647,16 @@
     </row>
     <row r="40" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B40" t="e" vm="37">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B40" t="e" vm="37">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="E40">
         <v>18.3</v>
@@ -3670,16 +3670,16 @@
     </row>
     <row r="41" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B41" t="e" vm="38">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B41" t="e" vm="38">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="E41">
         <v>19.2</v>
@@ -3693,16 +3693,16 @@
     </row>
     <row r="42" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B42" t="e" vm="39">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B42" t="e" vm="39">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="E42">
         <v>17.2</v>
@@ -3716,16 +3716,16 @@
     </row>
     <row r="43" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B43" t="e" vm="40">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B43" t="e" vm="40">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C43" s="2" t="s">
+      <c r="D43" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="E43">
         <v>18.7</v>
@@ -3739,16 +3739,16 @@
     </row>
     <row r="44" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B44" t="e" vm="41">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B44" t="e" vm="41">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="E44">
         <v>18.5</v>
@@ -3762,30 +3762,30 @@
     </row>
     <row r="45" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B45" t="e" vm="42">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B45" t="e" vm="42">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B46" t="e" vm="43">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B46" t="e" vm="43">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="E46">
         <v>19.399999999999999</v>
@@ -3799,16 +3799,16 @@
     </row>
     <row r="47" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B47" t="e" vm="44">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B47" t="e" vm="44">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C47" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="E47">
         <v>20.5</v>
@@ -3822,16 +3822,16 @@
     </row>
     <row r="48" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B48" t="e" vm="45">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B48" t="e" vm="45">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C48" s="2" t="s">
+      <c r="D48" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="E48">
         <v>20.3</v>
@@ -3845,16 +3845,16 @@
     </row>
     <row r="49" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49" t="e" vm="46">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B49" t="e" vm="46">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C49" s="2" t="s">
+      <c r="D49" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="E49">
         <v>17.8</v>
@@ -3868,16 +3868,16 @@
     </row>
     <row r="50" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B50" t="e" vm="47">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="B50" t="e" vm="47">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>151</v>
       </c>
       <c r="E50">
         <v>20.7</v>
@@ -3891,16 +3891,16 @@
     </row>
     <row r="51" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B51" t="e" vm="48">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B51" t="e" vm="48">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C51" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>154</v>
       </c>
       <c r="E51">
         <v>17.7</v>
@@ -3914,16 +3914,16 @@
     </row>
     <row r="52" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B52" t="e" vm="49">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B52" t="e" vm="49">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C52" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="E52">
         <v>19</v>
@@ -3937,16 +3937,16 @@
     </row>
     <row r="53" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B53" t="e" vm="50">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B53" t="e" vm="50">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C53" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>160</v>
       </c>
       <c r="E53">
         <v>19.399999999999999</v>
@@ -3960,16 +3960,16 @@
     </row>
     <row r="54" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B54" t="e" vm="51">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B54" t="e" vm="51">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="E54">
         <v>17.3</v>
@@ -3983,16 +3983,16 @@
     </row>
     <row r="55" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B55" t="e" vm="52">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B55" t="e" vm="52">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C55" s="2" t="s">
+      <c r="D55" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>166</v>
       </c>
       <c r="E55">
         <v>18.600000000000001</v>
@@ -4006,16 +4006,16 @@
     </row>
     <row r="56" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B56" t="e" vm="53">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B56" t="e" vm="53">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C56" s="2" t="s">
+      <c r="D56" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="E56">
         <v>18.3</v>
@@ -4029,16 +4029,16 @@
     </row>
     <row r="57" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B57" t="e" vm="54">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B57" t="e" vm="54">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C57" s="2" t="s">
+      <c r="D57" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>172</v>
       </c>
       <c r="E57">
         <v>18.3</v>
@@ -4052,16 +4052,16 @@
     </row>
     <row r="58" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B58" t="e" vm="55">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B58" t="e" vm="55">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C58" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>175</v>
       </c>
       <c r="E58">
         <v>18.3</v>
@@ -4075,16 +4075,16 @@
     </row>
     <row r="59" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B59" t="e" vm="56">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B59" t="e" vm="56">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C59" s="2" t="s">
+      <c r="D59" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="E59">
         <v>18.3</v>
@@ -4098,16 +4098,16 @@
     </row>
     <row r="60" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B60" t="e" vm="57">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B60" t="e" vm="57">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C60" s="2" t="s">
+      <c r="D60" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>181</v>
       </c>
       <c r="E60">
         <v>17.399999999999999</v>
@@ -4121,16 +4121,16 @@
     </row>
     <row r="61" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B61" t="e" vm="58">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B61" t="e" vm="58">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C61" s="2" t="s">
+      <c r="D61" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>184</v>
       </c>
       <c r="E61">
         <v>17.3</v>
@@ -4144,16 +4144,16 @@
     </row>
     <row r="62" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B62" t="e" vm="59">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B62" t="e" vm="59">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C62" s="2" t="s">
+      <c r="D62" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="E62">
         <v>19.2</v>
@@ -4167,13 +4167,13 @@
     </row>
     <row r="63" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B63" t="e" vm="60">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="B63" t="e" vm="60">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="D63" s="2">
         <v>0</v>
@@ -4190,16 +4190,16 @@
     </row>
     <row r="64" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B64" t="e" vm="61">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B64" t="e" vm="61">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C64" s="2" t="s">
+      <c r="D64" s="2" t="s">
         <v>191</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>192</v>
       </c>
       <c r="E64">
         <v>17.3</v>
@@ -4213,30 +4213,30 @@
     </row>
     <row r="65" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B65" t="e" vm="62">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B65" t="e" vm="62">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C65" s="2" t="s">
+      <c r="D65" s="2" t="s">
         <v>194</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B66" t="e" vm="63">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B66" t="e" vm="63">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C66" s="2" t="s">
+      <c r="D66" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="E66">
         <v>19.5</v>
@@ -4250,16 +4250,16 @@
     </row>
     <row r="67" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B67" t="e" vm="64">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B67" t="e" vm="64">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C67" s="2" t="s">
+      <c r="D67" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="E67">
         <v>18.7</v>
@@ -4273,16 +4273,16 @@
     </row>
     <row r="68" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B68" t="e" vm="65">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B68" t="e" vm="65">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C68" s="2" t="s">
+      <c r="D68" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>204</v>
       </c>
       <c r="E68">
         <v>18.2</v>
@@ -4296,16 +4296,16 @@
     </row>
     <row r="69" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B69" t="e" vm="66">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B69" t="e" vm="66">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C69" s="2" t="s">
+      <c r="D69" s="2" t="s">
         <v>206</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="E69">
         <v>17.3</v>
@@ -4319,30 +4319,30 @@
     </row>
     <row r="70" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B70" t="e" vm="67">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C70" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B70" t="e" vm="67">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C70" s="2" t="s">
+      <c r="D70" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B71" t="e" vm="68">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B71" t="e" vm="68">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C71" s="2" t="s">
+      <c r="D71" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="E71">
         <v>18.600000000000001</v>
@@ -4356,44 +4356,44 @@
     </row>
     <row r="72" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B72" t="e" vm="69">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C72" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B72" t="e" vm="69">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C72" s="2" t="s">
+      <c r="D72" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B73" t="e" vm="70">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B73" t="e" vm="70">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C73" s="2" t="s">
+      <c r="D73" s="2" t="s">
         <v>218</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B74" t="e" vm="71">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B74" t="e" vm="71">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C74" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>221</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>222</v>
       </c>
       <c r="E74">
         <v>18.3</v>
@@ -4407,16 +4407,16 @@
     </row>
     <row r="75" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B75" t="e" vm="72">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B75" t="e" vm="72">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>224</v>
-      </c>
       <c r="D75" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E75" s="2">
         <v>18.100000000000001</v>
@@ -4430,16 +4430,16 @@
     </row>
     <row r="76" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B76" t="e" vm="73">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B76" t="e" vm="73">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>226</v>
-      </c>
       <c r="D76" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E76">
         <v>18.5</v>
@@ -4453,44 +4453,44 @@
     </row>
     <row r="77" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B77" t="e" vm="74">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C77" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B77" t="e" vm="74">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C77" s="2" t="s">
+      <c r="D77" s="2" t="s">
         <v>228</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B78" t="e" vm="75">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C78" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B78" t="e" vm="75">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C78" s="2" t="s">
+      <c r="D78" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B79" t="e" vm="76">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="B79" t="e" vm="76">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C79" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>235</v>
       </c>
       <c r="E79">
         <v>18.3</v>
@@ -4504,44 +4504,44 @@
     </row>
     <row r="80" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B80" t="e" vm="77">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B80" t="e" vm="77">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C80" s="2" t="s">
+      <c r="D80" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B81" t="e" vm="78">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B81" t="e" vm="78">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C81" s="2" t="s">
+      <c r="D81" s="2" t="s">
         <v>240</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B82" t="e" vm="79">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B82" t="e" vm="79">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C82" s="2" t="s">
+      <c r="D82" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>244</v>
       </c>
       <c r="E82">
         <v>19.8</v>
@@ -4555,16 +4555,16 @@
     </row>
     <row r="83" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B83" t="e" vm="80">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B83" t="e" vm="80">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C83" s="2" t="s">
+      <c r="D83" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>247</v>
       </c>
       <c r="E83">
         <v>19.899999999999999</v>
@@ -4578,27 +4578,27 @@
     </row>
     <row r="84" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B84" t="e" vm="81">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C84" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B84" t="e" vm="81">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C84" s="2" t="s">
+      <c r="D84" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B85" t="e" vm="82">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="B85" t="e" vm="82">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>252</v>
       </c>
       <c r="D85" s="2">
         <v>0</v>
@@ -4615,30 +4615,30 @@
     </row>
     <row r="86" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B86" t="e" vm="83">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B86" t="e" vm="83">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C86" s="2" t="s">
+      <c r="D86" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B87" t="e" vm="84">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C87" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B87" t="e" vm="84">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C87" s="2" t="s">
+      <c r="D87" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="E87">
         <v>5</v>
@@ -4652,16 +4652,16 @@
     </row>
     <row r="88" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B88" t="e" vm="85">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C88" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="B88" t="e" vm="85">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C88" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>261</v>
       </c>
       <c r="E88">
         <v>18.600000000000001</v>
@@ -4675,30 +4675,30 @@
     </row>
     <row r="89" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B89" t="e" vm="86">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C89" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B89" t="e" vm="86">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C89" s="2" t="s">
+      <c r="D89" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B90" t="e" vm="87">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C90" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="B90" t="e" vm="87">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C90" s="2" t="s">
+      <c r="D90" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="E90">
         <v>18.399999999999999</v>
@@ -4712,30 +4712,30 @@
     </row>
     <row r="91" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B91" t="e" vm="88">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C91" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="B91" t="e" vm="88">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C91" s="2" t="s">
+      <c r="D91" s="2" t="s">
         <v>269</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B92" t="e" vm="89">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C92" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B92" t="e" vm="89">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C92" s="2" t="s">
+      <c r="D92" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>273</v>
       </c>
       <c r="E92">
         <v>19.5</v>
@@ -4749,16 +4749,16 @@
     </row>
     <row r="93" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B93" t="e" vm="90">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C93" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B93" t="e" vm="90">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C93" s="2" t="s">
+      <c r="D93" s="2" t="s">
         <v>275</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>276</v>
       </c>
       <c r="E93">
         <v>21</v>
@@ -4772,16 +4772,16 @@
     </row>
     <row r="94" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B94" t="e" vm="91">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C94" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="B94" t="e" vm="91">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C94" s="2" t="s">
+      <c r="D94" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>279</v>
       </c>
       <c r="E94">
         <v>20.7</v>
@@ -4795,16 +4795,16 @@
     </row>
     <row r="95" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B95" t="e" vm="92">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C95" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="B95" t="e" vm="92">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C95" s="2" t="s">
+      <c r="D95" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>282</v>
       </c>
       <c r="E95">
         <v>20.6</v>
@@ -4818,16 +4818,16 @@
     </row>
     <row r="96" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B96" t="s">
+        <v>95</v>
+      </c>
+      <c r="C96" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="B96" t="s">
-        <v>96</v>
-      </c>
-      <c r="C96" s="2" t="s">
+      <c r="D96" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>285</v>
       </c>
       <c r="E96">
         <v>20.3</v>
@@ -4841,13 +4841,13 @@
     </row>
     <row r="97" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B97" t="s">
+        <v>95</v>
+      </c>
+      <c r="C97" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="B97" t="s">
-        <v>96</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>287</v>
       </c>
       <c r="D97" s="2">
         <v>0</v>
@@ -4864,16 +4864,16 @@
     </row>
     <row r="98" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="B98" t="e" vm="93">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C98" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="B98" t="e" vm="93">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C98" s="2" t="s">
+      <c r="D98" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="E98">
         <v>20.9</v>
@@ -4887,10 +4887,10 @@
     </row>
     <row r="99" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E99">
         <v>17.100000000000001</v>
@@ -4904,10 +4904,10 @@
     </row>
     <row r="100" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E100">
         <v>16.899999999999999</v>
@@ -4921,10 +4921,10 @@
     </row>
     <row r="101" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E101">
         <v>17.7</v>

</xml_diff>